<commit_message>
Logit function check and try to estimate probit
This is a bit of a cheat because the scaling function was found using a polynomial trend line in Excel
</commit_message>
<xml_diff>
--- a/Student.xlsx
+++ b/Student.xlsx
@@ -1,23 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{291658D9-04DD-BA4C-9C58-8C5DA6F289A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{274FB7D9-5F55-464C-9F4E-49EBACC8B9A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="-7500" windowWidth="38400" windowHeight="23500" activeTab="3" xr2:uid="{A7CD8C95-85D1-1E4C-B771-A6F8EF459DDC}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14420" activeTab="4" xr2:uid="{A7CD8C95-85D1-1E4C-B771-A6F8EF459DDC}"/>
   </bookViews>
   <sheets>
-    <sheet name="Graphique1" sheetId="2" r:id="rId1"/>
-    <sheet name="Feuil1" sheetId="1" r:id="rId2"/>
+    <sheet name="Student graph" sheetId="2" r:id="rId1"/>
+    <sheet name="Student PDF" sheetId="1" r:id="rId2"/>
     <sheet name="Code size" sheetId="3" r:id="rId3"/>
-    <sheet name="Logit pour estimer probit" sheetId="4" r:id="rId4"/>
+    <sheet name="Logit to estimate probit" sheetId="4" r:id="rId4"/>
+    <sheet name="Graphique1" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">'Logit to estimate probit'!$B$53:$B$103</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Logit to estimate probit'!$C$53:$C$103</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,15 +44,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <si>
     <t>x</t>
   </si>
   <si>
     <t>k</t>
-  </si>
-  <si>
-    <t>Méthode</t>
   </si>
   <si>
     <t>c</t>
@@ -101,19 +103,10 @@
     <t>Student</t>
   </si>
   <si>
-    <t>Itération 1</t>
-  </si>
-  <si>
-    <t>Itération 2</t>
-  </si>
-  <si>
     <t>RemoveDividableFactors</t>
   </si>
   <si>
     <t>RemoveEvenFactors</t>
-  </si>
-  <si>
-    <t>Itération 3</t>
   </si>
   <si>
     <t>∞</t>
@@ -134,7 +127,25 @@
     <t>logit(P)</t>
   </si>
   <si>
-    <t>logit(P) * Racine(π/8)</t>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Iteration 1</t>
+  </si>
+  <si>
+    <t>Iteration 2</t>
+  </si>
+  <si>
+    <t>Iteration 3</t>
+  </si>
+  <si>
+    <t>Iteration 4</t>
+  </si>
+  <si>
+    <t>For error margins, scaled logit is a bad estimate for probit.</t>
+  </si>
+  <si>
+    <t>logit(P) * sqrt(π/8)</t>
   </si>
 </sst>
 </file>
@@ -147,7 +158,7 @@
     <numFmt numFmtId="166" formatCode="0.000000"/>
     <numFmt numFmtId="167" formatCode="0.000000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -164,6 +175,26 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -191,7 +222,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -205,14 +236,20 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -307,7 +344,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$B$2</c:f>
+              <c:f>'Student PDF'!$B$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -330,7 +367,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -522,7 +559,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$B$3:$B$63</c:f>
+              <c:f>'Student PDF'!$B$3:$B$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -724,7 +761,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$C$2</c:f>
+              <c:f>'Student PDF'!$C$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -747,7 +784,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -939,7 +976,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$C$3:$C$63</c:f>
+              <c:f>'Student PDF'!$C$3:$C$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -1141,7 +1178,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$D$2</c:f>
+              <c:f>'Student PDF'!$D$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1164,7 +1201,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -1356,7 +1393,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$D$3:$D$63</c:f>
+              <c:f>'Student PDF'!$D$3:$D$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -1558,7 +1595,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$E$2</c:f>
+              <c:f>'Student PDF'!$E$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1581,7 +1618,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -1773,7 +1810,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$E$3:$E$63</c:f>
+              <c:f>'Student PDF'!$E$3:$E$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -1975,7 +2012,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$F$2</c:f>
+              <c:f>'Student PDF'!$F$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1998,7 +2035,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -2190,7 +2227,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$F$3:$F$63</c:f>
+              <c:f>'Student PDF'!$F$3:$F$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -2392,7 +2429,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$G$2</c:f>
+              <c:f>'Student PDF'!$G$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2417,7 +2454,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -2609,7 +2646,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$G$3:$G$63</c:f>
+              <c:f>'Student PDF'!$G$3:$G$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -2811,7 +2848,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$H$2</c:f>
+              <c:f>'Student PDF'!$H$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2836,7 +2873,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -3028,7 +3065,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$H$3:$H$63</c:f>
+              <c:f>'Student PDF'!$H$3:$H$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -3230,7 +3267,7 @@
           <c:order val="7"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$I$2</c:f>
+              <c:f>'Student PDF'!$I$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3255,7 +3292,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -3447,7 +3484,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$I$3:$I$63</c:f>
+              <c:f>'Student PDF'!$I$3:$I$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -3649,7 +3686,7 @@
           <c:order val="8"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$J$2</c:f>
+              <c:f>'Student PDF'!$J$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3674,7 +3711,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -3866,7 +3903,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$J$3:$J$63</c:f>
+              <c:f>'Student PDF'!$J$3:$J$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -4068,7 +4105,7 @@
           <c:order val="9"/>
           <c:tx>
             <c:strRef>
-              <c:f>Feuil1!$K$2</c:f>
+              <c:f>'Student PDF'!$K$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4093,7 +4130,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Feuil1!$A$3:$A$63</c:f>
+              <c:f>'Student PDF'!$A$3:$A$63</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="61"/>
@@ -4285,7 +4322,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Feuil1!$K$3:$K$63</c:f>
+              <c:f>'Student PDF'!$K$3:$K$63</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="61"/>
@@ -4691,7 +4728,685 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-CA"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="12700" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="6"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-5.2694138575462048E-2"/>
+                  <c:y val="-2.3566454281269703E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="#,##0.000000000" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:sysClr val="windowText" lastClr="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Logit to estimate probit'!$B$53:$B$103</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="51"/>
+                <c:pt idx="0">
+                  <c:v>0.51</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.52</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.53</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.54</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.55000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.56000000000000005</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.56999999999999995</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.57999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.59</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.61</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.62</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.63</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.64</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.65</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.66</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.67</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.68</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.69</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.71</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.72</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.73</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.74</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.76</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.77</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.78</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.79</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.81</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.82</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.83</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.84</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.85</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.86</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.87</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.88</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.89</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.9</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.91</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.92</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.93</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.94</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.96</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.97</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.97499999999999998</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.98</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>0.995</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Logit to estimate probit'!$C$53:$C$103</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="51"/>
+                <c:pt idx="0">
+                  <c:v>0.62663913452498909</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.62658529330730339</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.62649542825445159</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.62636934380453213</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.62620676410011844</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.62600733087712346</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.62577060069151458</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.62549604143737314</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.62518302809673654</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.6248308376468622</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.62443864303341734</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.62400550609804195</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.62353036932496753</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.62301204624295092</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.62244921028445466</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.62184038186222546</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.62118391337217682</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.62047797176813557</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.6197205182751806</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.61890928470939011</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.6180417457468711</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.61711508632578982</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.61612616316080193</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.61507145908468641</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.61394702858621031</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.61274843245703348</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.61147065885223528</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.61010802724911362</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.60865407067031041</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.60710138999124796</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.60544147198475762</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.60366445967096583</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.60175885907472837</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.59971115990669355</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.59750533776880133</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.59512219021163282</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.59253843483268154</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.58972545833182743</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.58664753939902325</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.58325925295186498</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.57950155263477188</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.57529562341546225</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.57053276673771747</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.56505674749199553</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.55863057057379539</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.55086734357186706</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.54106450246968651</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.53498867327936173</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.52770908040868747</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.50626489621869231</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>0.48662024743359988</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3138-5442-9BD0-A33AF930F447}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="2063850000"/>
+        <c:axId val="2063908208"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="2063850000"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+          <c:min val="0.5"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2063908208"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="2063908208"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0.4"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2063850000"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+          <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+          <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -5247,8 +5962,532 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{D1279524-3F20-E644-915F-D13E0EDCDB7E}">
+  <sheetPr/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</chartsheet>
+</file>
+
+<file path=xl/chartsheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{A5F482BE-1A55-E34A-9D46-DF6031F6921B}">
   <sheetPr/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5259,7 +6498,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8673830" cy="6282447"/>
+    <xdr:ext cx="8676033" cy="6294783"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Graphique 1">
@@ -5496,6 +6735,39 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="8673830" cy="6282447"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Graphique 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8CE4DE39-C50B-80E1-B650-0AC9B17BC18E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5826,22 +7098,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B2">
@@ -5875,7 +7147,7 @@
         <v>89</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
@@ -9243,71 +10515,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
+      <c r="B1" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="E2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="H2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="K2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>30</v>
@@ -9348,7 +10620,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>133</v>
@@ -9389,7 +10661,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>29</v>
@@ -9430,7 +10702,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>146</v>
@@ -9471,7 +10743,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>307</v>
@@ -9512,7 +10784,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>81</v>
@@ -9553,7 +10825,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>39</v>
@@ -9594,7 +10866,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>133</v>
@@ -9635,7 +10907,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>44</v>
@@ -9676,7 +10948,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H12">
         <v>24</v>
@@ -9699,7 +10971,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H13">
         <v>22</v>
@@ -9713,7 +10985,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14">
         <v>58</v>
@@ -9754,7 +11026,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15">
         <v>74</v>
@@ -9795,7 +11067,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16">
         <v>71</v>
@@ -9809,7 +11081,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17">
         <v>72</v>
@@ -9841,7 +11113,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18">
         <v>86</v>
@@ -9957,2039 +11229,2217 @@
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="K1:M1"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15EA3DC0-928B-6544-A33C-0C895A9004BF}">
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:G106"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B2">
         <v>0</v>
       </c>
-      <c r="C2" t="e">
+      <c r="D2" t="e">
         <f>_xlfn.NORM.S.INV(B2)</f>
         <v>#NUM!</v>
       </c>
-      <c r="D2" t="e">
+      <c r="E2" t="e">
         <f>LN(B2/(1-B2))</f>
         <v>#NUM!</v>
       </c>
-      <c r="E2" t="e">
-        <f>D2*SQRT(0.125*PI())</f>
+      <c r="F2" t="e">
+        <f>E2*SQRT(0.125*PI())</f>
         <v>#NUM!</v>
       </c>
-      <c r="F2" s="3" t="e">
-        <f>(E2-C2)/C2</f>
+      <c r="G2" s="3" t="e">
+        <f>(F2-D2)/D2</f>
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B3">
         <v>0.01</v>
       </c>
-      <c r="C3">
-        <f t="shared" ref="C3:C66" si="0">_xlfn.NORM.S.INV(B3)</f>
+      <c r="D3">
+        <f t="shared" ref="D3:D66" si="0">_xlfn.NORM.S.INV(B3)</f>
         <v>-2.3263478740408408</v>
       </c>
-      <c r="D3">
-        <f t="shared" ref="D3:D66" si="1">LN(B3/(1-B3))</f>
+      <c r="E3">
+        <f t="shared" ref="E3:E66" si="1">LN(B3/(1-B3))</f>
         <v>-4.5951198501345898</v>
       </c>
-      <c r="E3">
-        <f t="shared" ref="E3:E66" si="2">D3*SQRT(0.125*PI())</f>
+      <c r="F3">
+        <f t="shared" ref="F3:F66" si="2">E3*SQRT(0.125*PI())</f>
         <v>-2.879564335416382</v>
       </c>
-      <c r="F3" s="3">
-        <f>(E3-C3)/C3</f>
+      <c r="G3" s="3">
+        <f>(F3-D3)/D3</f>
         <v>0.23780470132981887</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B4">
         <v>0.02</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <f t="shared" si="0"/>
         <v>-2.0537489106318225</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <f t="shared" si="1"/>
         <v>-3.8918202981106265</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <f t="shared" si="2"/>
         <v>-2.4388366997567363</v>
       </c>
-      <c r="F4" s="3">
-        <f t="shared" ref="F4:F67" si="3">(E4-C4)/C4</f>
+      <c r="G4" s="3">
+        <f t="shared" ref="G4:G67" si="3">(F4-D4)/D4</f>
         <v>0.18750480505742256</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B5">
         <v>0.03</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <f t="shared" si="0"/>
         <v>-1.8807936081512509</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <f t="shared" si="1"/>
         <v>-3.4760986898352733</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <f t="shared" si="2"/>
         <v>-2.1783218153372177</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="3">
         <f t="shared" si="3"/>
         <v>0.15819290638616421</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B6">
         <v>0.04</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <f t="shared" si="0"/>
         <v>-1.7506860712521695</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <f t="shared" si="1"/>
         <v>-3.1780538303479453</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <f t="shared" si="2"/>
         <v>-1.991549897362378</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="3">
         <f t="shared" si="3"/>
         <v>0.13758253410786084</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B7">
         <v>0.05</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <f t="shared" si="0"/>
         <v>-1.6448536269514726</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <f t="shared" si="1"/>
         <v>-2.9444389791664403</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <f t="shared" si="2"/>
         <v>-1.8451534995260594</v>
       </c>
-      <c r="F7" s="3">
+      <c r="G7" s="3">
         <f t="shared" si="3"/>
         <v>0.12177367596277681</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B8">
         <v>0.06</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <f t="shared" si="0"/>
         <v>-1.554773594596853</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <f t="shared" si="1"/>
         <v>-2.7515353130419489</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <f t="shared" si="2"/>
         <v>-1.7242690535791523</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G8" s="3">
         <f t="shared" si="3"/>
         <v>0.1090161677374311</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <f t="shared" si="0"/>
         <v>-1.4757910281791702</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <f t="shared" si="1"/>
         <v>-2.5866893440979424</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <f t="shared" si="2"/>
         <v>-1.6209671619006547</v>
       </c>
-      <c r="F9" s="3">
+      <c r="G9" s="3">
         <f t="shared" si="3"/>
         <v>9.8371741628354201E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B10">
         <v>0.08</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <f t="shared" si="0"/>
         <v>-1.4050715603096353</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <f t="shared" si="1"/>
         <v>-2.4423470353692043</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <f t="shared" si="2"/>
         <v>-1.5305140338294119</v>
       </c>
-      <c r="F10" s="3">
+      <c r="G10" s="3">
         <f t="shared" si="3"/>
         <v>8.9278352123313087E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B11">
         <v>0.09</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <f t="shared" si="0"/>
         <v>-1.3407550336902161</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <f t="shared" si="1"/>
         <v>-2.3136349291806306</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <f t="shared" si="2"/>
         <v>-1.4498556826645153</v>
       </c>
-      <c r="F11" s="3">
+      <c r="G11" s="3">
         <f t="shared" si="3"/>
         <v>8.1372544747430026E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B12">
         <v>0.1</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <f t="shared" si="0"/>
         <v>-1.2815515655446006</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <f t="shared" si="1"/>
         <v>-2.1972245773362191</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <f t="shared" si="2"/>
         <v>-1.3769063128162788</v>
       </c>
-      <c r="F12" s="3">
+      <c r="G12" s="3">
         <f t="shared" si="3"/>
         <v>7.4405704643774412E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B13">
         <v>0.11</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <f t="shared" si="0"/>
         <v>-1.2265281200366105</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <f t="shared" si="1"/>
         <v>-2.0907410969337694</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <f t="shared" si="2"/>
         <v>-1.3101776871268047</v>
       </c>
-      <c r="F13" s="3">
+      <c r="G13" s="3">
         <f t="shared" si="3"/>
         <v>6.820028479061481E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B14">
         <v>0.12</v>
       </c>
-      <c r="C14">
+      <c r="D14">
         <f t="shared" si="0"/>
         <v>-1.1749867920660904</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <f t="shared" si="1"/>
         <v>-1.9924301646902063</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <f t="shared" si="2"/>
         <v>-1.2485704465100429</v>
       </c>
-      <c r="F14" s="3">
+      <c r="G14" s="3">
         <f t="shared" si="3"/>
         <v>6.2625090716605797E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B15">
         <v>0.13</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <f t="shared" si="0"/>
         <v>-1.1263911290388013</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <f t="shared" si="1"/>
         <v>-1.900958761193047</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <f t="shared" si="2"/>
         <v>-1.1912492449285028</v>
       </c>
-      <c r="F15" s="3">
+      <c r="G15" s="3">
         <f t="shared" si="3"/>
         <v>5.7580456928001317E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B16">
         <v>0.14000000000000001</v>
       </c>
-      <c r="C16">
+      <c r="D16">
         <f t="shared" si="0"/>
         <v>-1.0803193408149565</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <f t="shared" si="1"/>
         <v>-1.8152899666382492</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <f t="shared" si="2"/>
         <v>-1.1375642892573501</v>
       </c>
-      <c r="F16" s="3">
+      <c r="G16" s="3">
         <f t="shared" si="3"/>
         <v>5.2988913814326348E-2</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17">
         <v>0.15</v>
       </c>
-      <c r="C17">
+      <c r="D17">
         <f t="shared" si="0"/>
         <v>-1.0364333894937898</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <f t="shared" si="1"/>
         <v>-1.7346010553881064</v>
       </c>
-      <c r="E17">
+      <c r="F17">
         <f t="shared" si="2"/>
         <v>-1.0870000126601502</v>
       </c>
-      <c r="F17" s="3">
+      <c r="G17" s="3">
         <f t="shared" si="3"/>
         <v>4.8789071906548596E-2</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18">
         <v>0.16</v>
       </c>
-      <c r="C18">
+      <c r="D18">
         <f t="shared" si="0"/>
         <v>-0.9944578832097497</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <f t="shared" si="1"/>
         <v>-1.6582280766035322</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <f t="shared" si="2"/>
         <v>-1.0391403456503485</v>
       </c>
-      <c r="F18" s="3">
+      <c r="G18" s="3">
         <f t="shared" si="3"/>
         <v>4.4931477938894723E-2</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19">
         <v>0.17</v>
       </c>
-      <c r="C19">
+      <c r="D19">
         <f t="shared" si="0"/>
         <v>-0.95416525314619549</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <f t="shared" si="1"/>
         <v>-1.5856272637403817</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <f t="shared" si="2"/>
         <v>-0.99364453307935674</v>
       </c>
-      <c r="F19" s="3">
+      <c r="G19" s="3">
         <f t="shared" si="3"/>
         <v>4.1375725853551183E-2</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20">
         <v>0.18</v>
       </c>
-      <c r="C20">
+      <c r="D20">
         <f t="shared" si="0"/>
         <v>-0.91536508784281501</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <f t="shared" si="1"/>
         <v>-1.5163474893680886</v>
       </c>
-      <c r="E20">
+      <c r="F20">
         <f t="shared" si="2"/>
         <v>-0.95022987275394522</v>
       </c>
-      <c r="F20" s="3">
+      <c r="G20" s="3">
         <f t="shared" si="3"/>
         <v>3.8088392679792846E-2</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21">
         <v>0.19</v>
       </c>
-      <c r="C21">
+      <c r="D21">
         <f t="shared" si="0"/>
         <v>-0.87789629505122846</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <f t="shared" si="1"/>
         <v>-1.4500101755059984</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <f t="shared" si="2"/>
         <v>-0.90865912610649868</v>
       </c>
-      <c r="F21" s="3">
+      <c r="G21" s="3">
         <f t="shared" si="3"/>
         <v>3.5041531931143531E-2</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22">
         <v>0.2</v>
       </c>
-      <c r="C22">
+      <c r="D22">
         <f t="shared" si="0"/>
         <v>-0.84162123357291452</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <f t="shared" si="1"/>
         <v>-1.3862943611198906</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <f t="shared" si="2"/>
         <v>-0.86873116063615907</v>
       </c>
-      <c r="F22" s="3">
+      <c r="G22" s="3">
         <f t="shared" si="3"/>
         <v>3.2211553109414114E-2</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23">
         <v>0.21</v>
       </c>
-      <c r="C23">
+      <c r="D23">
         <f t="shared" si="0"/>
         <v>-0.80642124701824058</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <f t="shared" si="1"/>
         <v>-1.3249254147435987</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <f t="shared" si="2"/>
         <v>-0.83027387659337726</v>
       </c>
-      <c r="F23" s="3">
+      <c r="G23" s="3">
         <f t="shared" si="3"/>
         <v>2.957837440832849E-2</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24">
         <v>0.22</v>
       </c>
-      <c r="C24">
+      <c r="D24">
         <f t="shared" si="0"/>
         <v>-0.77219321418868503</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <f t="shared" si="1"/>
         <v>-1.2656663733312759</v>
       </c>
-      <c r="E24">
+      <c r="F24">
         <f t="shared" si="2"/>
         <v>-0.79313877941046285</v>
       </c>
-      <c r="F24" s="3">
+      <c r="G24" s="3">
         <f t="shared" si="3"/>
         <v>2.7124772449320926E-2</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25">
         <v>0.23</v>
       </c>
-      <c r="C25">
+      <c r="D25">
         <f t="shared" si="0"/>
         <v>-0.73884684918521393</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <f t="shared" si="1"/>
         <v>-1.2083112059245342</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <f t="shared" si="2"/>
         <v>-0.75719675833097966</v>
       </c>
-      <c r="F25" s="3">
+      <c r="G25" s="3">
         <f t="shared" si="3"/>
         <v>2.4835876563595902E-2</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26">
         <v>0.24</v>
       </c>
-      <c r="C26">
+      <c r="D26">
         <f t="shared" si="0"/>
         <v>-0.7063025628400873</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <f t="shared" si="1"/>
         <v>-1.1526795099383855</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <f t="shared" si="2"/>
         <v>-0.72233476279984055</v>
       </c>
-      <c r="F26" s="3">
+      <c r="G26" s="3">
         <f t="shared" si="3"/>
         <v>2.2698770758082423E-2</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27">
         <v>0.25</v>
       </c>
-      <c r="C27">
+      <c r="D27">
         <f t="shared" si="0"/>
         <v>-0.67448975019608193</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <f t="shared" si="1"/>
         <v>-1.0986122886681098</v>
       </c>
-      <c r="E27">
+      <c r="F27">
         <f t="shared" si="2"/>
         <v>-0.68845315640813964</v>
       </c>
-      <c r="F27" s="3">
+      <c r="G27" s="3">
         <f t="shared" si="3"/>
         <v>2.0702177027891667E-2</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28">
         <v>0.26</v>
       </c>
-      <c r="C28">
+      <c r="D28">
         <f t="shared" si="0"/>
         <v>-0.64334540539291696</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <f t="shared" si="1"/>
         <v>-1.0459685551826876</v>
       </c>
-      <c r="E28">
+      <c r="F28">
         <f t="shared" si="2"/>
         <v>-0.65546358869896515</v>
       </c>
-      <c r="F28" s="3">
+      <c r="G28" s="3">
         <f t="shared" si="3"/>
         <v>1.88362009030703E-2</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29">
         <v>0.27</v>
       </c>
-      <c r="C29">
+      <c r="D29">
         <f t="shared" si="0"/>
         <v>-0.61281299101662734</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <f t="shared" si="1"/>
         <v>-0.99462257514406194</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <f t="shared" si="2"/>
         <v>-0.62328726736060058</v>
       </c>
-      <c r="F29" s="3">
+      <c r="G29" s="3">
         <f t="shared" si="3"/>
         <v>1.7092125163007593E-2</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30">
         <v>0.28000000000000003</v>
       </c>
-      <c r="C30">
+      <c r="D30">
         <f t="shared" si="0"/>
         <v>-0.58284150727121631</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <f t="shared" si="1"/>
         <v>-0.94446160884085117</v>
       </c>
-      <c r="E30">
+      <c r="F30">
         <f t="shared" si="2"/>
         <v>-0.59185354325599038</v>
       </c>
-      <c r="F30" s="3">
+      <c r="G30" s="3">
         <f t="shared" si="3"/>
         <v>1.5462241230840236E-2</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31">
         <v>0.28999999999999998</v>
       </c>
-      <c r="C31">
+      <c r="D31">
         <f t="shared" si="0"/>
         <v>-0.55338471955567303</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <f t="shared" si="1"/>
         <v>-0.89538404705484131</v>
       </c>
-      <c r="E31">
+      <c r="F31">
         <f t="shared" si="2"/>
         <v>-0.56109874225029976</v>
       </c>
-      <c r="F31" s="3">
+      <c r="G31" s="3">
         <f t="shared" si="3"/>
         <v>1.3939710335371242E-2</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32">
         <v>0.3</v>
       </c>
-      <c r="C32">
+      <c r="D32">
         <f t="shared" si="0"/>
         <v>-0.52440051270804089</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <f t="shared" si="1"/>
         <v>-0.84729786038720356</v>
       </c>
-      <c r="E32">
+      <c r="F32">
         <f t="shared" si="2"/>
         <v>-0.53096519347022852</v>
       </c>
-      <c r="F32" s="3">
+      <c r="G32" s="3">
         <f t="shared" si="3"/>
         <v>1.2518448405565367E-2</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33">
         <v>0.31</v>
       </c>
-      <c r="C33">
+      <c r="D33">
         <f t="shared" si="0"/>
         <v>-0.49585034734745354</v>
       </c>
-      <c r="D33">
+      <c r="E33">
         <f t="shared" si="1"/>
         <v>-0.80011930011211307</v>
       </c>
-      <c r="E33">
+      <c r="F33">
         <f t="shared" si="2"/>
         <v>-0.50140041518474732</v>
       </c>
-      <c r="F33" s="3">
+      <c r="G33" s="3">
         <f t="shared" si="3"/>
         <v>1.1193030048247045E-2</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34">
         <v>0.32</v>
       </c>
-      <c r="C34">
+      <c r="D34">
         <f t="shared" si="0"/>
         <v>-0.46769879911450829</v>
       </c>
-      <c r="D34">
+      <c r="E34">
         <f t="shared" si="1"/>
         <v>-0.75377180237638008</v>
       </c>
-      <c r="E34">
+      <c r="F34">
         <f t="shared" si="2"/>
         <v>-0.47235642811405121</v>
       </c>
-      <c r="F34" s="3">
+      <c r="G34" s="3">
         <f t="shared" si="3"/>
         <v>9.9586079937797195E-3</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35">
         <v>0.33</v>
       </c>
-      <c r="C35">
+      <c r="D35">
         <f t="shared" si="0"/>
         <v>-0.43991316567323374</v>
       </c>
-      <c r="D35">
+      <c r="E35">
         <f t="shared" si="1"/>
         <v>-0.70818505792448561</v>
       </c>
-      <c r="E35">
+      <c r="F35">
         <f t="shared" si="2"/>
         <v>-0.44378917246617711</v>
       </c>
-      <c r="F35" s="3">
+      <c r="G35" s="3">
         <f t="shared" si="3"/>
         <v>8.8108451744371118E-3</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B36">
         <v>0.34</v>
       </c>
-      <c r="C36">
+      <c r="D36">
         <f t="shared" si="0"/>
         <v>-0.41246312944140484</v>
       </c>
-      <c r="D36">
+      <c r="E36">
         <f t="shared" si="1"/>
         <v>-0.66329421741026395</v>
       </c>
-      <c r="E36">
+      <c r="F36">
         <f t="shared" si="2"/>
         <v>-0.41565800993995239</v>
       </c>
-      <c r="F36" s="3">
+      <c r="G36" s="3">
         <f t="shared" si="3"/>
         <v>7.7458571942523591E-3</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37">
         <v>0.35</v>
       </c>
-      <c r="C37">
+      <c r="D37">
         <f t="shared" si="0"/>
         <v>-0.38532046640756784</v>
       </c>
-      <c r="D37">
+      <c r="E37">
         <f t="shared" si="1"/>
         <v>-0.61903920840622351</v>
       </c>
-      <c r="E37">
+      <c r="F37">
         <f t="shared" si="2"/>
         <v>-0.38792529572405804</v>
       </c>
-      <c r="F37" s="3">
+      <c r="G37" s="3">
         <f t="shared" si="3"/>
         <v>6.7601634057376358E-3</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B38">
         <v>0.36</v>
       </c>
-      <c r="C38">
+      <c r="D38">
         <f t="shared" si="0"/>
         <v>-0.35845879325119384</v>
       </c>
-      <c r="D38">
+      <c r="E38">
         <f t="shared" si="1"/>
         <v>-0.5753641449035618</v>
       </c>
-      <c r="E38">
+      <c r="F38">
         <f t="shared" si="2"/>
         <v>-0.36055600845603897</v>
       </c>
-      <c r="F38" s="3">
+      <c r="G38" s="3">
         <f t="shared" si="3"/>
         <v>5.8506451629308492E-3</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39">
         <v>0.37</v>
       </c>
-      <c r="C39">
+      <c r="D39">
         <f t="shared" si="0"/>
         <v>-0.33185334643681658</v>
       </c>
-      <c r="D39">
+      <c r="E39">
         <f t="shared" si="1"/>
         <v>-0.53221681374730823</v>
       </c>
-      <c r="E39">
+      <c r="F39">
         <f t="shared" si="2"/>
         <v>-0.33351742839325593</v>
       </c>
-      <c r="F39" s="3">
+      <c r="G39" s="3">
         <f t="shared" si="3"/>
         <v>5.0145100970262176E-3</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B40">
         <v>0.38</v>
       </c>
-      <c r="C40">
+      <c r="D40">
         <f t="shared" si="0"/>
         <v>-0.30548078809939727</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <f t="shared" si="1"/>
         <v>-0.48954822531870579</v>
       </c>
-      <c r="E40">
+      <c r="F40">
         <f t="shared" si="2"/>
         <v>-0.30677885584482389</v>
       </c>
-      <c r="F40" s="3">
+      <c r="G40" s="3">
         <f t="shared" si="3"/>
         <v>4.2492614789387609E-3</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41">
         <v>0.39</v>
       </c>
-      <c r="C41">
+      <c r="D41">
         <f t="shared" si="0"/>
         <v>-0.27931903444745415</v>
       </c>
-      <c r="D41">
+      <c r="E41">
         <f t="shared" si="1"/>
         <v>-0.44731221804366478</v>
       </c>
-      <c r="E41">
+      <c r="F41">
         <f t="shared" si="2"/>
         <v>-0.28031136333403928</v>
       </c>
-      <c r="F41" s="3">
+      <c r="G41" s="3">
         <f t="shared" si="3"/>
         <v>3.5526719063315522E-3</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B42">
         <v>0.4</v>
       </c>
-      <c r="C42">
+      <c r="D42">
         <f t="shared" si="0"/>
         <v>-0.25334710313579978</v>
       </c>
-      <c r="D42">
+      <c r="E42">
         <f t="shared" si="1"/>
         <v>-0.40546510810816427</v>
       </c>
-      <c r="E42">
+      <c r="F42">
         <f t="shared" si="2"/>
         <v>-0.25408757609005994</v>
       </c>
-      <c r="F42" s="3">
+      <c r="G42" s="3">
         <f t="shared" si="3"/>
         <v>2.9227606911425888E-3</v>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43">
         <v>0.41</v>
       </c>
-      <c r="C43">
+      <c r="D43">
         <f t="shared" si="0"/>
         <v>-0.2275449766411495</v>
       </c>
-      <c r="D43">
+      <c r="E43">
         <f t="shared" si="1"/>
         <v>-0.36396537720141192</v>
       </c>
-      <c r="E43">
+      <c r="F43">
         <f t="shared" si="2"/>
         <v>-0.22808147636994908</v>
       </c>
-      <c r="F43" s="3">
+      <c r="G43" s="3">
         <f t="shared" si="3"/>
         <v>2.3577744352742212E-3</v>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B44">
         <v>0.42</v>
       </c>
-      <c r="C44">
+      <c r="D44">
         <f t="shared" si="0"/>
         <v>-0.20189347914185088</v>
       </c>
-      <c r="D44">
+      <c r="E44">
         <f t="shared" si="1"/>
         <v>-0.32277339226305118</v>
       </c>
-      <c r="E44">
+      <c r="F44">
         <f t="shared" si="2"/>
         <v>-0.20226822783628176</v>
       </c>
-      <c r="F44" s="3">
+      <c r="G44" s="3">
         <f t="shared" si="3"/>
         <v>1.8561703727319621E-3</v>
       </c>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B45">
         <v>0.43</v>
       </c>
-      <c r="C45">
+      <c r="D45">
         <f t="shared" si="0"/>
         <v>-0.17637416478086138</v>
       </c>
-      <c r="D45">
+      <c r="E45">
         <f t="shared" si="1"/>
         <v>-0.28185115214098788</v>
       </c>
-      <c r="E45">
+      <c r="F45">
         <f t="shared" si="2"/>
         <v>-0.176624016798481</v>
       </c>
-      <c r="F45" s="3">
+      <c r="G45" s="3">
         <f t="shared" si="3"/>
         <v>1.4166021306468272E-3</v>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B46">
         <v>0.44</v>
       </c>
-      <c r="C46">
+      <c r="D46">
         <f t="shared" si="0"/>
         <v>-0.15096921549677725</v>
       </c>
-      <c r="D46">
+      <c r="E46">
         <f t="shared" si="1"/>
         <v>-0.2411620568168881</v>
       </c>
-      <c r="E46">
+      <c r="F46">
         <f t="shared" si="2"/>
         <v>-0.15112590759634487</v>
       </c>
-      <c r="F46" s="3">
+      <c r="G46" s="3">
         <f t="shared" si="3"/>
         <v>1.0379076227693778E-3</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B47">
         <v>0.45</v>
       </c>
-      <c r="C47">
+      <c r="D47">
         <f t="shared" si="0"/>
         <v>-0.12566134685507402</v>
       </c>
-      <c r="D47">
+      <c r="E47">
         <f t="shared" si="1"/>
         <v>-0.20067069546215124</v>
       </c>
-      <c r="E47">
+      <c r="F47">
         <f t="shared" si="2"/>
         <v>-0.12575170978382377</v>
       </c>
-      <c r="F47" s="3">
+      <c r="G47" s="3">
         <f t="shared" si="3"/>
         <v>7.1909883994773966E-4</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B48">
         <v>0.46</v>
       </c>
-      <c r="C48">
+      <c r="D48">
         <f t="shared" si="0"/>
         <v>-0.10043372051146976</v>
       </c>
-      <c r="D48">
+      <c r="E48">
         <f t="shared" si="1"/>
         <v>-0.16034265007517937</v>
       </c>
-      <c r="E48">
+      <c r="F48">
         <f t="shared" si="2"/>
         <v>-0.10047985507692726</v>
       </c>
-      <c r="F48" s="3">
+      <c r="G48" s="3">
         <f t="shared" si="3"/>
         <v>4.5935334489808949E-4</v>
       </c>
     </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B49">
         <v>0.47</v>
       </c>
-      <c r="C49">
+      <c r="D49">
         <f t="shared" si="0"/>
         <v>-7.5269862099829901E-2</v>
       </c>
-      <c r="D49">
+      <c r="E49">
         <f t="shared" si="1"/>
         <v>-0.12014431184206334</v>
       </c>
-      <c r="E49">
+      <c r="F49">
         <f t="shared" si="2"/>
         <v>-7.5289282274850017E-2</v>
       </c>
-      <c r="F49" s="3">
+      <c r="G49" s="3">
         <f t="shared" si="3"/>
         <v>2.5800731499094244E-4</v>
       </c>
     </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B50">
         <v>0.48</v>
       </c>
-      <c r="C50">
+      <c r="D50">
         <f t="shared" si="0"/>
         <v>-5.0153583464733656E-2</v>
       </c>
-      <c r="D50">
+      <c r="E50">
         <f t="shared" si="1"/>
         <v>-8.0042707673536495E-2</v>
       </c>
-      <c r="E50">
+      <c r="F50">
         <f t="shared" si="2"/>
         <v>-5.0159328558127575E-2</v>
       </c>
-      <c r="F50" s="3">
+      <c r="G50" s="3">
         <f t="shared" si="3"/>
         <v>1.1455000813568591E-4</v>
       </c>
     </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B51">
         <v>0.49</v>
       </c>
-      <c r="C51">
+      <c r="D51">
         <f t="shared" si="0"/>
         <v>-2.506890825871106E-2</v>
       </c>
-      <c r="D51">
+      <c r="E51">
         <f t="shared" si="1"/>
         <v>-4.0005334613699248E-2</v>
       </c>
-      <c r="E51">
+      <c r="F51">
         <f t="shared" si="2"/>
         <v>-2.5069625719693196E-2</v>
       </c>
-      <c r="F51" s="3">
+      <c r="G51" s="3">
         <f t="shared" si="3"/>
         <v>2.8619554339223177E-5</v>
       </c>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B52">
         <v>0.5</v>
       </c>
-      <c r="C52">
+      <c r="D52">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D52">
+      <c r="E52">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E52">
+      <c r="F52">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F52" s="3">
+      <c r="G52" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B53">
         <v>0.51</v>
       </c>
       <c r="C53">
+        <f>D53/E53</f>
+        <v>0.62663913452498909</v>
+      </c>
+      <c r="D53">
         <f t="shared" si="0"/>
         <v>2.506890825871106E-2</v>
       </c>
-      <c r="D53">
+      <c r="E53">
         <f t="shared" si="1"/>
         <v>4.0005334613699206E-2</v>
       </c>
-      <c r="E53">
+      <c r="F53">
         <f t="shared" si="2"/>
         <v>2.5069625719693168E-2</v>
       </c>
-      <c r="F53" s="3">
+      <c r="G53" s="3">
         <f t="shared" si="3"/>
         <v>2.8619554338116003E-5</v>
       </c>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B54">
         <v>0.52</v>
       </c>
       <c r="C54">
+        <f t="shared" ref="C54:C103" si="4">D54/E54</f>
+        <v>0.62658529330730339</v>
+      </c>
+      <c r="D54">
         <f t="shared" si="0"/>
         <v>5.0153583464733656E-2</v>
       </c>
-      <c r="D54">
+      <c r="E54">
         <f t="shared" si="1"/>
         <v>8.0042707673536564E-2</v>
       </c>
-      <c r="E54">
+      <c r="F54">
         <f t="shared" si="2"/>
         <v>5.0159328558127624E-2</v>
       </c>
-      <c r="F54" s="3">
+      <c r="G54" s="3">
         <f t="shared" si="3"/>
         <v>1.1455000813665439E-4</v>
       </c>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B55">
         <v>0.53</v>
       </c>
       <c r="C55">
+        <f t="shared" si="4"/>
+        <v>0.62649542825445159</v>
+      </c>
+      <c r="D55">
         <f t="shared" si="0"/>
         <v>7.5269862099829901E-2</v>
       </c>
-      <c r="D55">
+      <c r="E55">
         <f t="shared" si="1"/>
         <v>0.12014431184206341</v>
       </c>
-      <c r="E55">
+      <c r="F55">
         <f t="shared" si="2"/>
         <v>7.5289282274850058E-2</v>
       </c>
-      <c r="F55" s="3">
+      <c r="G55" s="3">
         <f t="shared" si="3"/>
         <v>2.580073149914956E-4</v>
       </c>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B56">
         <v>0.54</v>
       </c>
       <c r="C56">
+        <f t="shared" si="4"/>
+        <v>0.62636934380453213</v>
+      </c>
+      <c r="D56">
         <f t="shared" si="0"/>
         <v>0.10043372051146988</v>
       </c>
-      <c r="D56">
+      <c r="E56">
         <f t="shared" si="1"/>
         <v>0.16034265007517948</v>
       </c>
-      <c r="E56">
+      <c r="F56">
         <f t="shared" si="2"/>
         <v>0.10047985507692733</v>
       </c>
-      <c r="F56" s="3">
+      <c r="G56" s="3">
         <f t="shared" si="3"/>
         <v>4.5935334489753622E-4</v>
       </c>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B57">
         <v>0.55000000000000004</v>
       </c>
       <c r="C57">
+        <f t="shared" si="4"/>
+        <v>0.62620676410011844</v>
+      </c>
+      <c r="D57">
         <f t="shared" si="0"/>
         <v>0.12566134685507416</v>
       </c>
-      <c r="D57">
+      <c r="E57">
         <f t="shared" si="1"/>
         <v>0.20067069546215141</v>
       </c>
-      <c r="E57">
+      <c r="F57">
         <f t="shared" si="2"/>
         <v>0.12575170978382386</v>
       </c>
-      <c r="F57" s="3">
+      <c r="G57" s="3">
         <f t="shared" si="3"/>
         <v>7.1909883994729709E-4</v>
       </c>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B58">
         <v>0.56000000000000005</v>
       </c>
       <c r="C58">
+        <f t="shared" si="4"/>
+        <v>0.62600733087712346</v>
+      </c>
+      <c r="D58">
         <f t="shared" si="0"/>
         <v>0.15096921549677741</v>
       </c>
-      <c r="D58">
+      <c r="E58">
         <f t="shared" si="1"/>
         <v>0.24116205681688824</v>
       </c>
-      <c r="E58">
+      <c r="F58">
         <f t="shared" si="2"/>
         <v>0.15112590759634495</v>
       </c>
-      <c r="F58" s="3">
+      <c r="G58" s="3">
         <f t="shared" si="3"/>
         <v>1.037907622768825E-3</v>
       </c>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B59">
         <v>0.56999999999999995</v>
       </c>
       <c r="C59">
+        <f t="shared" si="4"/>
+        <v>0.62577060069151458</v>
+      </c>
+      <c r="D59">
         <f t="shared" si="0"/>
         <v>0.17637416478086121</v>
       </c>
-      <c r="D59">
+      <c r="E59">
         <f t="shared" si="1"/>
         <v>0.28185115214098749</v>
       </c>
-      <c r="E59">
+      <c r="F59">
         <f t="shared" si="2"/>
         <v>0.17662401679848075</v>
       </c>
-      <c r="F59" s="3">
+      <c r="G59" s="3">
         <f t="shared" si="3"/>
         <v>1.4166021306463565E-3</v>
       </c>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B60">
         <v>0.57999999999999996</v>
       </c>
       <c r="C60">
+        <f t="shared" si="4"/>
+        <v>0.62549604143737314</v>
+      </c>
+      <c r="D60">
         <f t="shared" si="0"/>
         <v>0.20189347914185077</v>
       </c>
-      <c r="D60">
+      <c r="E60">
         <f t="shared" si="1"/>
         <v>0.32277339226305085</v>
       </c>
-      <c r="E60">
+      <c r="F60">
         <f t="shared" si="2"/>
         <v>0.20226822783628154</v>
       </c>
-      <c r="F60" s="3">
+      <c r="G60" s="3">
         <f t="shared" si="3"/>
         <v>1.8561703727314133E-3</v>
       </c>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B61">
         <v>0.59</v>
       </c>
       <c r="C61">
+        <f t="shared" si="4"/>
+        <v>0.62518302809673654</v>
+      </c>
+      <c r="D61">
         <f t="shared" si="0"/>
         <v>0.22754497664114934</v>
       </c>
-      <c r="D61">
+      <c r="E61">
         <f t="shared" si="1"/>
         <v>0.36396537720141148</v>
       </c>
-      <c r="E61">
+      <c r="F61">
         <f t="shared" si="2"/>
         <v>0.2280814763699488</v>
       </c>
-      <c r="F61" s="3">
+      <c r="G61" s="3">
         <f t="shared" si="3"/>
         <v>2.357774435273735E-3</v>
       </c>
     </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B62">
         <v>0.6</v>
       </c>
       <c r="C62">
+        <f t="shared" si="4"/>
+        <v>0.6248308376468622</v>
+      </c>
+      <c r="D62">
         <f t="shared" si="0"/>
         <v>0.25334710313579978</v>
       </c>
-      <c r="D62">
+      <c r="E62">
         <f t="shared" si="1"/>
         <v>0.40546510810816422</v>
       </c>
-      <c r="E62">
+      <c r="F62">
         <f t="shared" si="2"/>
         <v>0.25408757609005994</v>
       </c>
-      <c r="F62" s="3">
+      <c r="G62" s="3">
         <f t="shared" si="3"/>
         <v>2.9227606911425888E-3</v>
       </c>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B63">
         <v>0.61</v>
       </c>
       <c r="C63">
+        <f t="shared" si="4"/>
+        <v>0.62443864303341734</v>
+      </c>
+      <c r="D63">
         <f t="shared" si="0"/>
         <v>0.27931903444745415</v>
       </c>
-      <c r="D63">
+      <c r="E63">
         <f t="shared" si="1"/>
         <v>0.44731221804366483</v>
       </c>
-      <c r="E63">
+      <c r="F63">
         <f t="shared" si="2"/>
         <v>0.28031136333403933</v>
       </c>
-      <c r="F63" s="3">
+      <c r="G63" s="3">
         <f t="shared" si="3"/>
         <v>3.5526719063317508E-3</v>
       </c>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B64">
         <v>0.62</v>
       </c>
       <c r="C64">
+        <f t="shared" si="4"/>
+        <v>0.62400550609804195</v>
+      </c>
+      <c r="D64">
         <f t="shared" si="0"/>
         <v>0.30548078809939727</v>
       </c>
-      <c r="D64">
+      <c r="E64">
         <f t="shared" si="1"/>
         <v>0.48954822531870579</v>
       </c>
-      <c r="E64">
+      <c r="F64">
         <f t="shared" si="2"/>
         <v>0.30677885584482389</v>
       </c>
-      <c r="F64" s="3">
+      <c r="G64" s="3">
         <f t="shared" si="3"/>
         <v>4.2492614789387609E-3</v>
       </c>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B65">
         <v>0.63</v>
       </c>
       <c r="C65">
+        <f t="shared" si="4"/>
+        <v>0.62353036932496753</v>
+      </c>
+      <c r="D65">
         <f t="shared" si="0"/>
         <v>0.33185334643681658</v>
       </c>
-      <c r="D65">
+      <c r="E65">
         <f t="shared" si="1"/>
         <v>0.53221681374730823</v>
       </c>
-      <c r="E65">
+      <c r="F65">
         <f t="shared" si="2"/>
         <v>0.33351742839325593</v>
       </c>
-      <c r="F65" s="3">
+      <c r="G65" s="3">
         <f t="shared" si="3"/>
         <v>5.0145100970262176E-3</v>
       </c>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B66">
         <v>0.64</v>
       </c>
       <c r="C66">
+        <f t="shared" si="4"/>
+        <v>0.62301204624295092</v>
+      </c>
+      <c r="D66">
         <f t="shared" si="0"/>
         <v>0.35845879325119384</v>
       </c>
-      <c r="D66">
+      <c r="E66">
         <f t="shared" si="1"/>
         <v>0.57536414490356191</v>
       </c>
-      <c r="E66">
+      <c r="F66">
         <f t="shared" si="2"/>
         <v>0.36055600845603908</v>
       </c>
-      <c r="F66" s="3">
+      <c r="G66" s="3">
         <f t="shared" si="3"/>
         <v>5.8506451629311588E-3</v>
       </c>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B67">
         <v>0.65</v>
       </c>
       <c r="C67">
-        <f t="shared" ref="C67:C104" si="4">_xlfn.NORM.S.INV(B67)</f>
+        <f t="shared" si="4"/>
+        <v>0.62244921028445466</v>
+      </c>
+      <c r="D67">
+        <f t="shared" ref="D67:D104" si="5">_xlfn.NORM.S.INV(B67)</f>
         <v>0.38532046640756784</v>
       </c>
-      <c r="D67">
-        <f t="shared" ref="D67:D104" si="5">LN(B67/(1-B67))</f>
+      <c r="E67">
+        <f t="shared" ref="E67:E104" si="6">LN(B67/(1-B67))</f>
         <v>0.61903920840622362</v>
       </c>
-      <c r="E67">
-        <f t="shared" ref="E67:E104" si="6">D67*SQRT(0.125*PI())</f>
+      <c r="F67">
+        <f t="shared" ref="F67:F104" si="7">E67*SQRT(0.125*PI())</f>
         <v>0.38792529572405809</v>
       </c>
-      <c r="F67" s="3">
+      <c r="G67" s="3">
         <f t="shared" si="3"/>
         <v>6.7601634057377798E-3</v>
       </c>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B68">
         <v>0.66</v>
       </c>
       <c r="C68">
         <f t="shared" si="4"/>
-        <v>0.41246312944140473</v>
+        <v>0.62184038186222546</v>
       </c>
       <c r="D68">
         <f t="shared" si="5"/>
-        <v>0.66329421741026429</v>
+        <v>0.41246312944140473</v>
       </c>
       <c r="E68">
         <f t="shared" si="6"/>
+        <v>0.66329421741026429</v>
+      </c>
+      <c r="F68">
+        <f t="shared" si="7"/>
         <v>0.41565800993995256</v>
       </c>
-      <c r="F68" s="3">
-        <f t="shared" ref="F68:F104" si="7">(E68-C68)/C68</f>
+      <c r="G68" s="3">
+        <f t="shared" ref="G68:G104" si="8">(F68-D68)/D68</f>
         <v>7.7458571942530339E-3</v>
       </c>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B69">
         <v>0.67</v>
       </c>
       <c r="C69">
         <f t="shared" si="4"/>
-        <v>0.43991316567323396</v>
+        <v>0.62118391337217682</v>
       </c>
       <c r="D69">
         <f t="shared" si="5"/>
-        <v>0.70818505792448605</v>
+        <v>0.43991316567323396</v>
       </c>
       <c r="E69">
         <f t="shared" si="6"/>
+        <v>0.70818505792448605</v>
+      </c>
+      <c r="F69">
+        <f t="shared" si="7"/>
         <v>0.44378917246617738</v>
       </c>
-      <c r="F69" s="3">
-        <f t="shared" si="7"/>
+      <c r="G69" s="3">
+        <f t="shared" si="8"/>
         <v>8.8108451744372332E-3</v>
       </c>
     </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B70">
         <v>0.68</v>
       </c>
       <c r="C70">
         <f t="shared" si="4"/>
-        <v>0.46769879911450835</v>
+        <v>0.62047797176813557</v>
       </c>
       <c r="D70">
         <f t="shared" si="5"/>
-        <v>0.75377180237638031</v>
+        <v>0.46769879911450835</v>
       </c>
       <c r="E70">
         <f t="shared" si="6"/>
+        <v>0.75377180237638031</v>
+      </c>
+      <c r="F70">
+        <f t="shared" si="7"/>
         <v>0.47235642811405137</v>
       </c>
-      <c r="F70" s="3">
-        <f t="shared" si="7"/>
+      <c r="G70" s="3">
+        <f t="shared" si="8"/>
         <v>9.9586079937799554E-3</v>
       </c>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B71">
         <v>0.69</v>
       </c>
       <c r="C71">
         <f t="shared" si="4"/>
-        <v>0.49585034734745331</v>
+        <v>0.6197205182751806</v>
       </c>
       <c r="D71">
         <f t="shared" si="5"/>
-        <v>0.80011930011211285</v>
+        <v>0.49585034734745331</v>
       </c>
       <c r="E71">
         <f t="shared" si="6"/>
+        <v>0.80011930011211285</v>
+      </c>
+      <c r="F71">
+        <f t="shared" si="7"/>
         <v>0.50140041518474721</v>
       </c>
-      <c r="F71" s="3">
-        <f t="shared" si="7"/>
+      <c r="G71" s="3">
+        <f t="shared" si="8"/>
         <v>1.1193030048247274E-2</v>
       </c>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B72">
         <v>0.7</v>
       </c>
       <c r="C72">
         <f t="shared" si="4"/>
-        <v>0.52440051270804078</v>
+        <v>0.61890928470939011</v>
       </c>
       <c r="D72">
         <f t="shared" si="5"/>
-        <v>0.84729786038720345</v>
+        <v>0.52440051270804078</v>
       </c>
       <c r="E72">
         <f t="shared" si="6"/>
+        <v>0.84729786038720345</v>
+      </c>
+      <c r="F72">
+        <f t="shared" si="7"/>
         <v>0.53096519347022852</v>
       </c>
-      <c r="F72" s="3">
-        <f t="shared" si="7"/>
+      <c r="G72" s="3">
+        <f t="shared" si="8"/>
         <v>1.2518448405565583E-2</v>
       </c>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B73">
         <v>0.71</v>
       </c>
       <c r="C73">
         <f t="shared" si="4"/>
-        <v>0.5533847195556727</v>
+        <v>0.6180417457468711</v>
       </c>
       <c r="D73">
         <f t="shared" si="5"/>
-        <v>0.89538404705484131</v>
+        <v>0.5533847195556727</v>
       </c>
       <c r="E73">
         <f t="shared" si="6"/>
+        <v>0.89538404705484131</v>
+      </c>
+      <c r="F73">
+        <f t="shared" si="7"/>
         <v>0.56109874225029976</v>
       </c>
-      <c r="F73" s="3">
-        <f t="shared" si="7"/>
+      <c r="G73" s="3">
+        <f t="shared" si="8"/>
         <v>1.3939710335371853E-2</v>
       </c>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B74">
         <v>0.72</v>
       </c>
       <c r="C74">
         <f t="shared" si="4"/>
-        <v>0.58284150727121631</v>
+        <v>0.61711508632578982</v>
       </c>
       <c r="D74">
         <f t="shared" si="5"/>
-        <v>0.94446160884085129</v>
+        <v>0.58284150727121631</v>
       </c>
       <c r="E74">
         <f t="shared" si="6"/>
+        <v>0.94446160884085129</v>
+      </c>
+      <c r="F74">
+        <f t="shared" si="7"/>
         <v>0.59185354325599038</v>
       </c>
-      <c r="F74" s="3">
-        <f t="shared" si="7"/>
+      <c r="G74" s="3">
+        <f t="shared" si="8"/>
         <v>1.5462241230840236E-2</v>
       </c>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B75">
         <v>0.73</v>
       </c>
       <c r="C75">
         <f t="shared" si="4"/>
-        <v>0.61281299101662734</v>
+        <v>0.61612616316080193</v>
       </c>
       <c r="D75">
         <f t="shared" si="5"/>
-        <v>0.99462257514406194</v>
+        <v>0.61281299101662734</v>
       </c>
       <c r="E75">
         <f t="shared" si="6"/>
+        <v>0.99462257514406194</v>
+      </c>
+      <c r="F75">
+        <f t="shared" si="7"/>
         <v>0.62328726736060058</v>
       </c>
-      <c r="F75" s="3">
-        <f t="shared" si="7"/>
+      <c r="G75" s="3">
+        <f t="shared" si="8"/>
         <v>1.7092125163007593E-2</v>
       </c>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B76">
         <v>0.74</v>
       </c>
       <c r="C76">
         <f t="shared" si="4"/>
-        <v>0.64334540539291696</v>
+        <v>0.61507145908468641</v>
       </c>
       <c r="D76">
         <f t="shared" si="5"/>
-        <v>1.0459685551826876</v>
+        <v>0.64334540539291696</v>
       </c>
       <c r="E76">
         <f t="shared" si="6"/>
+        <v>1.0459685551826876</v>
+      </c>
+      <c r="F76">
+        <f t="shared" si="7"/>
         <v>0.65546358869896515</v>
       </c>
-      <c r="F76" s="3">
-        <f t="shared" si="7"/>
+      <c r="G76" s="3">
+        <f t="shared" si="8"/>
         <v>1.88362009030703E-2</v>
       </c>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B77">
         <v>0.75</v>
       </c>
       <c r="C77">
         <f t="shared" si="4"/>
-        <v>0.67448975019608193</v>
+        <v>0.61394702858621031</v>
       </c>
       <c r="D77">
         <f t="shared" si="5"/>
-        <v>1.0986122886681098</v>
+        <v>0.67448975019608193</v>
       </c>
       <c r="E77">
         <f t="shared" si="6"/>
+        <v>1.0986122886681098</v>
+      </c>
+      <c r="F77">
+        <f t="shared" si="7"/>
         <v>0.68845315640813964</v>
       </c>
-      <c r="F77" s="3">
-        <f t="shared" si="7"/>
+      <c r="G77" s="3">
+        <f t="shared" si="8"/>
         <v>2.0702177027891667E-2</v>
       </c>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B78">
         <v>0.76</v>
       </c>
       <c r="C78">
         <f t="shared" si="4"/>
-        <v>0.7063025628400873</v>
+        <v>0.61274843245703348</v>
       </c>
       <c r="D78">
         <f t="shared" si="5"/>
-        <v>1.1526795099383855</v>
+        <v>0.7063025628400873</v>
       </c>
       <c r="E78">
         <f t="shared" si="6"/>
+        <v>1.1526795099383855</v>
+      </c>
+      <c r="F78">
+        <f t="shared" si="7"/>
         <v>0.72233476279984055</v>
       </c>
-      <c r="F78" s="3">
-        <f t="shared" si="7"/>
+      <c r="G78" s="3">
+        <f t="shared" si="8"/>
         <v>2.2698770758082423E-2</v>
       </c>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B79">
         <v>0.77</v>
       </c>
       <c r="C79">
         <f t="shared" si="4"/>
-        <v>0.73884684918521393</v>
+        <v>0.61147065885223528</v>
       </c>
       <c r="D79">
         <f t="shared" si="5"/>
-        <v>1.2083112059245342</v>
+        <v>0.73884684918521393</v>
       </c>
       <c r="E79">
         <f t="shared" si="6"/>
+        <v>1.2083112059245342</v>
+      </c>
+      <c r="F79">
+        <f t="shared" si="7"/>
         <v>0.75719675833097966</v>
       </c>
-      <c r="F79" s="3">
-        <f t="shared" si="7"/>
+      <c r="G79" s="3">
+        <f t="shared" si="8"/>
         <v>2.4835876563595902E-2</v>
       </c>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B80">
         <v>0.78</v>
       </c>
       <c r="C80">
         <f t="shared" si="4"/>
-        <v>0.77219321418868503</v>
+        <v>0.61010802724911362</v>
       </c>
       <c r="D80">
         <f t="shared" si="5"/>
-        <v>1.2656663733312761</v>
+        <v>0.77219321418868503</v>
       </c>
       <c r="E80">
         <f t="shared" si="6"/>
+        <v>1.2656663733312761</v>
+      </c>
+      <c r="F80">
+        <f t="shared" si="7"/>
         <v>0.79313877941046296</v>
       </c>
-      <c r="F80" s="3">
-        <f t="shared" si="7"/>
+      <c r="G80" s="3">
+        <f t="shared" si="8"/>
         <v>2.7124772449321072E-2</v>
       </c>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B81">
         <v>0.79</v>
       </c>
       <c r="C81">
         <f t="shared" si="4"/>
-        <v>0.80642124701824058</v>
+        <v>0.60865407067031041</v>
       </c>
       <c r="D81">
         <f t="shared" si="5"/>
-        <v>1.3249254147435987</v>
+        <v>0.80642124701824058</v>
       </c>
       <c r="E81">
         <f t="shared" si="6"/>
+        <v>1.3249254147435987</v>
+      </c>
+      <c r="F81">
+        <f t="shared" si="7"/>
         <v>0.83027387659337726</v>
       </c>
-      <c r="F81" s="3">
-        <f t="shared" si="7"/>
+      <c r="G81" s="3">
+        <f t="shared" si="8"/>
         <v>2.957837440832849E-2</v>
       </c>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B82">
         <v>0.8</v>
       </c>
       <c r="C82">
         <f t="shared" si="4"/>
-        <v>0.84162123357291474</v>
+        <v>0.60710138999124796</v>
       </c>
       <c r="D82">
         <f t="shared" si="5"/>
-        <v>1.3862943611198908</v>
+        <v>0.84162123357291474</v>
       </c>
       <c r="E82">
         <f t="shared" si="6"/>
+        <v>1.3862943611198908</v>
+      </c>
+      <c r="F82">
+        <f t="shared" si="7"/>
         <v>0.86873116063615918</v>
       </c>
-      <c r="F82" s="3">
-        <f t="shared" si="7"/>
+      <c r="G82" s="3">
+        <f t="shared" si="8"/>
         <v>3.2211553109413968E-2</v>
       </c>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B83">
         <v>0.81</v>
       </c>
       <c r="C83">
         <f t="shared" si="4"/>
-        <v>0.87789629505122857</v>
+        <v>0.60544147198475762</v>
       </c>
       <c r="D83">
         <f t="shared" si="5"/>
-        <v>1.4500101755059986</v>
+        <v>0.87789629505122857</v>
       </c>
       <c r="E83">
         <f t="shared" si="6"/>
+        <v>1.4500101755059986</v>
+      </c>
+      <c r="F83">
+        <f t="shared" si="7"/>
         <v>0.90865912610649879</v>
       </c>
-      <c r="F83" s="3">
-        <f t="shared" si="7"/>
+      <c r="G83" s="3">
+        <f t="shared" si="8"/>
         <v>3.5041531931143524E-2</v>
       </c>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B84">
         <v>0.82</v>
       </c>
       <c r="C84">
         <f t="shared" si="4"/>
-        <v>0.91536508784281256</v>
+        <v>0.60366445967096583</v>
       </c>
       <c r="D84">
         <f t="shared" si="5"/>
-        <v>1.5163474893680882</v>
+        <v>0.91536508784281256</v>
       </c>
       <c r="E84">
         <f t="shared" si="6"/>
+        <v>1.5163474893680882</v>
+      </c>
+      <c r="F84">
+        <f t="shared" si="7"/>
         <v>0.95022987275394499</v>
       </c>
-      <c r="F84" s="3">
-        <f t="shared" si="7"/>
+      <c r="G84" s="3">
+        <f t="shared" si="8"/>
         <v>3.8088392679795371E-2</v>
       </c>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B85">
         <v>0.83</v>
       </c>
       <c r="C85">
         <f t="shared" si="4"/>
-        <v>0.95416525314619549</v>
+        <v>0.60175885907472837</v>
       </c>
       <c r="D85">
         <f t="shared" si="5"/>
-        <v>1.5856272637403817</v>
+        <v>0.95416525314619549</v>
       </c>
       <c r="E85">
         <f t="shared" si="6"/>
+        <v>1.5856272637403817</v>
+      </c>
+      <c r="F85">
+        <f t="shared" si="7"/>
         <v>0.99364453307935674</v>
       </c>
-      <c r="F85" s="3">
-        <f t="shared" si="7"/>
+      <c r="G85" s="3">
+        <f t="shared" si="8"/>
         <v>4.1375725853551183E-2</v>
       </c>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B86">
         <v>0.84</v>
       </c>
       <c r="C86">
         <f t="shared" si="4"/>
-        <v>0.9944578832097497</v>
+        <v>0.59971115990669355</v>
       </c>
       <c r="D86">
         <f t="shared" si="5"/>
-        <v>1.6582280766035322</v>
+        <v>0.9944578832097497</v>
       </c>
       <c r="E86">
         <f t="shared" si="6"/>
+        <v>1.6582280766035322</v>
+      </c>
+      <c r="F86">
+        <f t="shared" si="7"/>
         <v>1.0391403456503485</v>
       </c>
-      <c r="F86" s="3">
-        <f t="shared" si="7"/>
+      <c r="G86" s="3">
+        <f t="shared" si="8"/>
         <v>4.4931477938894723E-2</v>
       </c>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B87">
         <v>0.85</v>
       </c>
       <c r="C87">
         <f t="shared" si="4"/>
-        <v>1.0364333894937898</v>
+        <v>0.59750533776880133</v>
       </c>
       <c r="D87">
         <f t="shared" si="5"/>
-        <v>1.7346010553881064</v>
+        <v>1.0364333894937898</v>
       </c>
       <c r="E87">
         <f t="shared" si="6"/>
+        <v>1.7346010553881064</v>
+      </c>
+      <c r="F87">
+        <f t="shared" si="7"/>
         <v>1.0870000126601502</v>
       </c>
-      <c r="F87" s="3">
-        <f t="shared" si="7"/>
+      <c r="G87" s="3">
+        <f t="shared" si="8"/>
         <v>4.8789071906548596E-2</v>
       </c>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B88">
         <v>0.86</v>
       </c>
       <c r="C88">
         <f t="shared" si="4"/>
-        <v>1.0803193408149565</v>
+        <v>0.59512219021163282</v>
       </c>
       <c r="D88">
         <f t="shared" si="5"/>
-        <v>1.8152899666382489</v>
+        <v>1.0803193408149565</v>
       </c>
       <c r="E88">
         <f t="shared" si="6"/>
+        <v>1.8152899666382489</v>
+      </c>
+      <c r="F88">
+        <f t="shared" si="7"/>
         <v>1.1375642892573499</v>
       </c>
-      <c r="F88" s="3">
-        <f t="shared" si="7"/>
+      <c r="G88" s="3">
+        <f t="shared" si="8"/>
         <v>5.2988913814326147E-2</v>
       </c>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B89">
         <v>0.87</v>
       </c>
       <c r="C89">
         <f t="shared" si="4"/>
-        <v>1.1263911290388013</v>
+        <v>0.59253843483268154</v>
       </c>
       <c r="D89">
         <f t="shared" si="5"/>
-        <v>1.900958761193047</v>
+        <v>1.1263911290388013</v>
       </c>
       <c r="E89">
         <f t="shared" si="6"/>
+        <v>1.900958761193047</v>
+      </c>
+      <c r="F89">
+        <f t="shared" si="7"/>
         <v>1.1912492449285028</v>
       </c>
-      <c r="F89" s="3">
-        <f t="shared" si="7"/>
+      <c r="G89" s="3">
+        <f t="shared" si="8"/>
         <v>5.7580456928001317E-2</v>
       </c>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B90">
         <v>0.88</v>
       </c>
       <c r="C90">
         <f t="shared" si="4"/>
-        <v>1.1749867920660904</v>
+        <v>0.58972545833182743</v>
       </c>
       <c r="D90">
         <f t="shared" si="5"/>
-        <v>1.9924301646902063</v>
+        <v>1.1749867920660904</v>
       </c>
       <c r="E90">
         <f t="shared" si="6"/>
+        <v>1.9924301646902063</v>
+      </c>
+      <c r="F90">
+        <f t="shared" si="7"/>
         <v>1.2485704465100429</v>
       </c>
-      <c r="F90" s="3">
-        <f t="shared" si="7"/>
+      <c r="G90" s="3">
+        <f t="shared" si="8"/>
         <v>6.2625090716605797E-2</v>
       </c>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B91">
         <v>0.89</v>
       </c>
       <c r="C91">
         <f t="shared" si="4"/>
-        <v>1.2265281200366105</v>
+        <v>0.58664753939902325</v>
       </c>
       <c r="D91">
         <f t="shared" si="5"/>
-        <v>2.0907410969337694</v>
+        <v>1.2265281200366105</v>
       </c>
       <c r="E91">
         <f t="shared" si="6"/>
+        <v>2.0907410969337694</v>
+      </c>
+      <c r="F91">
+        <f t="shared" si="7"/>
         <v>1.3101776871268047</v>
       </c>
-      <c r="F91" s="3">
-        <f t="shared" si="7"/>
+      <c r="G91" s="3">
+        <f t="shared" si="8"/>
         <v>6.820028479061481E-2</v>
       </c>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B92">
         <v>0.9</v>
       </c>
       <c r="C92">
         <f t="shared" si="4"/>
-        <v>1.2815515655446006</v>
+        <v>0.58325925295186498</v>
       </c>
       <c r="D92">
         <f t="shared" si="5"/>
-        <v>2.1972245773362196</v>
+        <v>1.2815515655446006</v>
       </c>
       <c r="E92">
         <f t="shared" si="6"/>
+        <v>2.1972245773362196</v>
+      </c>
+      <c r="F92">
+        <f t="shared" si="7"/>
         <v>1.3769063128162793</v>
       </c>
-      <c r="F92" s="3">
-        <f t="shared" si="7"/>
+      <c r="G92" s="3">
+        <f t="shared" si="8"/>
         <v>7.4405704643774759E-2</v>
       </c>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B93">
         <v>0.91</v>
       </c>
       <c r="C93">
         <f t="shared" si="4"/>
-        <v>1.3407550336902161</v>
+        <v>0.57950155263477188</v>
       </c>
       <c r="D93">
         <f t="shared" si="5"/>
-        <v>2.3136349291806311</v>
+        <v>1.3407550336902161</v>
       </c>
       <c r="E93">
         <f t="shared" si="6"/>
+        <v>2.3136349291806311</v>
+      </c>
+      <c r="F93">
+        <f t="shared" si="7"/>
         <v>1.4498556826645155</v>
       </c>
-      <c r="F93" s="3">
-        <f t="shared" si="7"/>
+      <c r="G93" s="3">
+        <f t="shared" si="8"/>
         <v>8.1372544747430192E-2</v>
       </c>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B94">
         <v>0.92</v>
       </c>
       <c r="C94">
         <f t="shared" si="4"/>
-        <v>1.4050715603096329</v>
+        <v>0.57529562341546225</v>
       </c>
       <c r="D94">
         <f t="shared" si="5"/>
-        <v>2.4423470353692052</v>
+        <v>1.4050715603096329</v>
       </c>
       <c r="E94">
         <f t="shared" si="6"/>
+        <v>2.4423470353692052</v>
+      </c>
+      <c r="F94">
+        <f t="shared" si="7"/>
         <v>1.5305140338294123</v>
       </c>
-      <c r="F94" s="3">
-        <f t="shared" si="7"/>
+      <c r="G94" s="3">
+        <f t="shared" si="8"/>
         <v>8.9278352123315294E-2</v>
       </c>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B95">
         <v>0.93</v>
       </c>
       <c r="C95">
         <f t="shared" si="4"/>
-        <v>1.4757910281791713</v>
+        <v>0.57053276673771747</v>
       </c>
       <c r="D95">
         <f t="shared" si="5"/>
-        <v>2.5866893440979433</v>
+        <v>1.4757910281791713</v>
       </c>
       <c r="E95">
         <f t="shared" si="6"/>
+        <v>2.5866893440979433</v>
+      </c>
+      <c r="F95">
+        <f t="shared" si="7"/>
         <v>1.6209671619006554</v>
       </c>
-      <c r="F95" s="3">
-        <f t="shared" si="7"/>
+      <c r="G95" s="3">
+        <f t="shared" si="8"/>
         <v>9.8371741628353826E-2</v>
       </c>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B96">
         <v>0.94</v>
       </c>
       <c r="C96">
         <f t="shared" si="4"/>
-        <v>1.5547735945968528</v>
+        <v>0.56505674749199553</v>
       </c>
       <c r="D96">
         <f t="shared" si="5"/>
-        <v>2.751535313041948</v>
+        <v>1.5547735945968528</v>
       </c>
       <c r="E96">
         <f t="shared" si="6"/>
+        <v>2.751535313041948</v>
+      </c>
+      <c r="F96">
+        <f t="shared" si="7"/>
         <v>1.7242690535791518</v>
       </c>
-      <c r="F96" s="3">
-        <f t="shared" si="7"/>
+      <c r="G96" s="3">
+        <f t="shared" si="8"/>
         <v>0.10901616773743097</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97">
-        <f t="shared" ref="A97:A101" si="8">2*(1-B97)</f>
+        <f t="shared" ref="A97:A101" si="9">2*(1-B97)</f>
         <v>0.10000000000000009</v>
       </c>
       <c r="B97">
@@ -11997,22 +13447,26 @@
       </c>
       <c r="C97">
         <f t="shared" si="4"/>
-        <v>1.6448536269514715</v>
+        <v>0.55863057057379539</v>
       </c>
       <c r="D97">
         <f t="shared" si="5"/>
-        <v>2.9444389791664394</v>
+        <v>1.6448536269514715</v>
       </c>
       <c r="E97">
         <f t="shared" si="6"/>
+        <v>2.9444389791664394</v>
+      </c>
+      <c r="F97">
+        <f t="shared" si="7"/>
         <v>1.845153499526059</v>
       </c>
-      <c r="F97" s="3">
-        <f t="shared" si="7"/>
+      <c r="G97" s="3">
+        <f t="shared" si="8"/>
         <v>0.1217736759627773</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98">
         <f>2*(1-B98)</f>
         <v>8.0000000000000071E-2</v>
@@ -12022,24 +13476,28 @@
       </c>
       <c r="C98">
         <f t="shared" si="4"/>
-        <v>1.7506860712521695</v>
+        <v>0.55086734357186706</v>
       </c>
       <c r="D98">
         <f t="shared" si="5"/>
-        <v>3.1780538303479449</v>
+        <v>1.7506860712521695</v>
       </c>
       <c r="E98">
         <f t="shared" si="6"/>
+        <v>3.1780538303479449</v>
+      </c>
+      <c r="F98">
+        <f t="shared" si="7"/>
         <v>1.9915498973623778</v>
       </c>
-      <c r="F98" s="3">
-        <f t="shared" si="7"/>
+      <c r="G98" s="3">
+        <f t="shared" si="8"/>
         <v>0.13758253410786073</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>6.0000000000000053E-2</v>
       </c>
       <c r="B99">
@@ -12047,24 +13505,28 @@
       </c>
       <c r="C99">
         <f t="shared" si="4"/>
-        <v>1.8807936081512504</v>
+        <v>0.54106450246968651</v>
       </c>
       <c r="D99">
         <f t="shared" si="5"/>
-        <v>3.4760986898352719</v>
+        <v>1.8807936081512504</v>
       </c>
       <c r="E99">
         <f t="shared" si="6"/>
+        <v>3.4760986898352719</v>
+      </c>
+      <c r="F99">
+        <f t="shared" si="7"/>
         <v>2.1783218153372172</v>
       </c>
-      <c r="F99" s="3">
-        <f t="shared" si="7"/>
+      <c r="G99" s="3">
+        <f t="shared" si="8"/>
         <v>0.15819290638616426</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>5.0000000000000044E-2</v>
       </c>
       <c r="B100">
@@ -12072,24 +13534,28 @@
       </c>
       <c r="C100">
         <f t="shared" si="4"/>
-        <v>1.9599639845400536</v>
+        <v>0.53498867327936173</v>
       </c>
       <c r="D100">
         <f t="shared" si="5"/>
-        <v>3.6635616461296454</v>
+        <v>1.9599639845400536</v>
       </c>
       <c r="E100">
         <f t="shared" si="6"/>
+        <v>3.6635616461296454</v>
+      </c>
+      <c r="F100">
+        <f t="shared" si="7"/>
         <v>2.2957968020105652</v>
       </c>
-      <c r="F100" s="3">
-        <f t="shared" si="7"/>
+      <c r="G100" s="3">
+        <f t="shared" si="8"/>
         <v>0.17134642275037609</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>4.0000000000000036E-2</v>
       </c>
       <c r="B101">
@@ -12097,22 +13563,26 @@
       </c>
       <c r="C101">
         <f t="shared" si="4"/>
-        <v>2.0537489106318221</v>
+        <v>0.52770908040868747</v>
       </c>
       <c r="D101">
         <f t="shared" si="5"/>
-        <v>3.8918202981106256</v>
+        <v>2.0537489106318221</v>
       </c>
       <c r="E101">
         <f t="shared" si="6"/>
+        <v>3.8918202981106256</v>
+      </c>
+      <c r="F101">
+        <f t="shared" si="7"/>
         <v>2.4388366997567354</v>
       </c>
-      <c r="F101" s="3">
-        <f t="shared" si="7"/>
+      <c r="G101" s="3">
+        <f t="shared" si="8"/>
         <v>0.18750480505742237</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102">
         <f>2*(1-B102)</f>
         <v>2.0000000000000018E-2</v>
@@ -12122,22 +13592,26 @@
       </c>
       <c r="C102">
         <f t="shared" si="4"/>
-        <v>2.3263478740408408</v>
+        <v>0.50626489621869231</v>
       </c>
       <c r="D102">
         <f t="shared" si="5"/>
-        <v>4.5951198501345889</v>
+        <v>2.3263478740408408</v>
       </c>
       <c r="E102">
         <f t="shared" si="6"/>
+        <v>4.5951198501345889</v>
+      </c>
+      <c r="F102">
+        <f t="shared" si="7"/>
         <v>2.8795643354163811</v>
       </c>
-      <c r="F102" s="3">
-        <f t="shared" si="7"/>
+      <c r="G102" s="3">
+        <f t="shared" si="8"/>
         <v>0.23780470132981851</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103">
         <f>2*(1-B103)</f>
         <v>1.0000000000000009E-2</v>
@@ -12147,43 +13621,61 @@
       </c>
       <c r="C103">
         <f t="shared" si="4"/>
-        <v>2.5758293035488999</v>
+        <v>0.48662024743359988</v>
       </c>
       <c r="D103">
         <f t="shared" si="5"/>
-        <v>5.2933048247244914</v>
+        <v>2.5758293035488999</v>
       </c>
       <c r="E103">
         <f t="shared" si="6"/>
+        <v>5.2933048247244914</v>
+      </c>
+      <c r="F103">
+        <f t="shared" si="7"/>
         <v>3.3170868849737754</v>
       </c>
-      <c r="F103" s="3">
-        <f t="shared" si="7"/>
+      <c r="G103" s="3">
+        <f t="shared" si="8"/>
         <v>0.28777434141446917</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B104">
         <v>1</v>
       </c>
-      <c r="C104" t="e">
-        <f t="shared" si="4"/>
-        <v>#NUM!</v>
-      </c>
       <c r="D104" t="e">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>#NUM!</v>
       </c>
       <c r="E104" t="e">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="F104" s="3" t="e">
+      <c r="F104" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
+      <c r="G104" s="3" t="e">
+        <f t="shared" si="8"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A106" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B106" s="12"/>
+      <c r="C106" s="12"/>
+      <c r="D106" s="12"/>
+      <c r="E106" s="12"/>
+      <c r="F106" s="12"/>
+      <c r="G106" s="12"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A106:G106"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Inverse normal distribution support, added erf and erf^-1
Cumulative mode is now supported on non-standard normal distributions. The inverse will need optimizations (hint: 2000 iterations is overkill).
</commit_message>
<xml_diff>
--- a/Student.xlsx
+++ b/Student.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{274FB7D9-5F55-464C-9F4E-49EBACC8B9A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15D7EBF7-02E5-5440-95A6-CC730981DF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14420" activeTab="4" xr2:uid="{A7CD8C95-85D1-1E4C-B771-A6F8EF459DDC}"/>
+    <workbookView xWindow="25600" yWindow="-7500" windowWidth="38400" windowHeight="23500" activeTab="4" xr2:uid="{A7CD8C95-85D1-1E4C-B771-A6F8EF459DDC}"/>
   </bookViews>
   <sheets>
     <sheet name="Student graph" sheetId="2" r:id="rId1"/>
@@ -19,10 +19,6 @@
     <sheet name="Logit to estimate probit" sheetId="4" r:id="rId4"/>
     <sheet name="Graphique1" sheetId="5" r:id="rId5"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'Logit to estimate probit'!$B$53:$B$103</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'Logit to estimate probit'!$C$53:$C$103</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -240,17 +236,17 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -301,8 +297,8 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="fr-CA" b="1"/>
-              <a:t>Distributions de Student</a:t>
+              <a:rPr lang="fr-CA" sz="1400" b="1"/>
+              <a:t>Student Distributions</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -4572,7 +4568,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1"/>
                 </a:solidFill>
@@ -4629,7 +4625,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1"/>
                 </a:solidFill>
@@ -4670,7 +4666,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
@@ -4743,6 +4739,33 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="fr-CA" b="1"/>
+              <a:t>Scaling</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="fr-CA" b="1" baseline="0"/>
+              <a:t> to apply to logit(p) to look like probit(p)</a:t>
+            </a:r>
+            <a:endParaRPr lang="fr-CA" b="1"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4758,7 +4781,7 @@
           <a:pPr>
             <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:ea typeface="+mn-ea"/>
@@ -4819,8 +4842,8 @@
             <c:trendlineLbl>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-5.2694138575462048E-2"/>
-                  <c:y val="-2.3566454281269703E-2"/>
+                  <c:x val="-2.5252166574627356E-2"/>
+                  <c:y val="-3.244277269668968E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:numFmt formatCode="#,##0.000000000" sourceLinked="0"/>
@@ -4838,7 +4861,7 @@
                   <a:pPr>
                     <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
-                        <a:sysClr val="windowText" lastClr="000000"/>
+                        <a:schemeClr val="tx1"/>
                       </a:solidFill>
                       <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                       <a:ea typeface="+mn-ea"/>
@@ -4852,10 +4875,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'Logit to estimate probit'!$B$53:$B$103</c:f>
+              <c:f>'Logit to estimate probit'!$B$53:$B$106</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="51"/>
+                <c:ptCount val="54"/>
                 <c:pt idx="0">
                   <c:v>0.51</c:v>
                 </c:pt>
@@ -4992,21 +5015,30 @@
                   <c:v>0.95</c:v>
                 </c:pt>
                 <c:pt idx="45">
+                  <c:v>0.95499999999999996</c:v>
+                </c:pt>
+                <c:pt idx="46">
                   <c:v>0.96</c:v>
                 </c:pt>
-                <c:pt idx="46">
+                <c:pt idx="47">
+                  <c:v>0.96499999999999997</c:v>
+                </c:pt>
+                <c:pt idx="48">
                   <c:v>0.97</c:v>
                 </c:pt>
-                <c:pt idx="47">
+                <c:pt idx="49">
                   <c:v>0.97499999999999998</c:v>
                 </c:pt>
-                <c:pt idx="48">
+                <c:pt idx="50">
                   <c:v>0.98</c:v>
                 </c:pt>
-                <c:pt idx="49">
+                <c:pt idx="51">
+                  <c:v>0.98499999999999999</c:v>
+                </c:pt>
+                <c:pt idx="52">
                   <c:v>0.99</c:v>
                 </c:pt>
-                <c:pt idx="50">
+                <c:pt idx="53">
                   <c:v>0.995</c:v>
                 </c:pt>
               </c:numCache>
@@ -5014,10 +5046,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Logit to estimate probit'!$C$53:$C$103</c:f>
+              <c:f>'Logit to estimate probit'!$C$53:$C$106</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="51"/>
+                <c:ptCount val="54"/>
                 <c:pt idx="0">
                   <c:v>0.62663913452498909</c:v>
                 </c:pt>
@@ -5154,21 +5186,30 @@
                   <c:v>0.55863057057379539</c:v>
                 </c:pt>
                 <c:pt idx="45">
+                  <c:v>0.55494946009714197</c:v>
+                </c:pt>
+                <c:pt idx="46">
                   <c:v>0.55086734357186706</c:v>
                 </c:pt>
-                <c:pt idx="46">
+                <c:pt idx="47">
+                  <c:v>0.54628605188867885</c:v>
+                </c:pt>
+                <c:pt idx="48">
                   <c:v>0.54106450246968651</c:v>
                 </c:pt>
-                <c:pt idx="47">
+                <c:pt idx="49">
                   <c:v>0.53498867327936173</c:v>
                 </c:pt>
-                <c:pt idx="48">
+                <c:pt idx="50">
                   <c:v>0.52770908040868747</c:v>
                 </c:pt>
-                <c:pt idx="49">
+                <c:pt idx="51">
+                  <c:v>0.51859074145320205</c:v>
+                </c:pt>
+                <c:pt idx="52">
                   <c:v>0.50626489621869231</c:v>
                 </c:pt>
-                <c:pt idx="50">
+                <c:pt idx="53">
                   <c:v>0.48662024743359988</c:v>
                 </c:pt>
               </c:numCache>
@@ -5215,18 +5256,15 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
+        <c:numFmt formatCode="#,##0.00" sourceLinked="0"/>
+        <c:majorTickMark val="cross"/>
+        <c:minorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -5237,9 +5275,9 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000"/>
+                  <a:schemeClr val="tx1"/>
                 </a:solidFill>
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:ea typeface="+mn-ea"/>
@@ -5252,12 +5290,13 @@
         <c:crossAx val="2063908208"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
+        <c:majorUnit val="0.1"/>
       </c:valAx>
       <c:valAx>
         <c:axId val="2063908208"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:min val="0.4"/>
+          <c:min val="0.45"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -5275,18 +5314,15 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
+        <c:numFmt formatCode="#,##0.00" sourceLinked="0"/>
+        <c:majorTickMark val="cross"/>
+        <c:minorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -5297,9 +5333,9 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000"/>
+                  <a:schemeClr val="tx1"/>
                 </a:solidFill>
                 <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                 <a:ea typeface="+mn-ea"/>
@@ -5312,11 +5348,14 @@
         <c:crossAx val="2063850000"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
+        <c:majorUnit val="0.05"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
         <a:ln>
-          <a:noFill/>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
         </a:ln>
         <a:effectLst/>
       </c:spPr>
@@ -5354,7 +5393,7 @@
       <a:pPr>
         <a:defRPr>
           <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
+            <a:schemeClr val="tx1"/>
           </a:solidFill>
           <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
           <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
@@ -6498,7 +6537,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8676033" cy="6294783"/>
+    <xdr:ext cx="8673830" cy="6282447"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Graphique 1">
@@ -7098,22 +7137,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B2">
@@ -10515,26 +10554,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11" t="s">
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11" t="s">
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11" t="s">
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -11236,7 +11275,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15EA3DC0-928B-6544-A33C-0C895A9004BF}">
-  <dimension ref="A1:G106"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
@@ -12367,7 +12406,7 @@
         <v>0.52</v>
       </c>
       <c r="C54">
-        <f t="shared" ref="C54:C103" si="4">D54/E54</f>
+        <f t="shared" ref="C54:C106" si="4">D54/E54</f>
         <v>0.62658529330730339</v>
       </c>
       <c r="D54">
@@ -12696,15 +12735,15 @@
         <v>0.62244921028445466</v>
       </c>
       <c r="D67">
-        <f t="shared" ref="D67:D104" si="5">_xlfn.NORM.S.INV(B67)</f>
+        <f t="shared" ref="D67:D107" si="5">_xlfn.NORM.S.INV(B67)</f>
         <v>0.38532046640756784</v>
       </c>
       <c r="E67">
-        <f t="shared" ref="E67:E104" si="6">LN(B67/(1-B67))</f>
+        <f t="shared" ref="E67:E107" si="6">LN(B67/(1-B67))</f>
         <v>0.61903920840622362</v>
       </c>
       <c r="F67">
-        <f t="shared" ref="F67:F104" si="7">E67*SQRT(0.125*PI())</f>
+        <f t="shared" ref="F67:F107" si="7">E67*SQRT(0.125*PI())</f>
         <v>0.38792529572405809</v>
       </c>
       <c r="G67" s="3">
@@ -12733,7 +12772,7 @@
         <v>0.41565800993995256</v>
       </c>
       <c r="G68" s="3">
-        <f t="shared" ref="G68:G104" si="8">(F68-D68)/D68</f>
+        <f t="shared" ref="G68:G107" si="8">(F68-D68)/D68</f>
         <v>7.7458571942530339E-3</v>
       </c>
     </row>
@@ -13439,7 +13478,7 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97">
-        <f t="shared" ref="A97:A101" si="9">2*(1-B97)</f>
+        <f t="shared" ref="A97:A104" si="9">2*(1-B97)</f>
         <v>0.10000000000000009</v>
       </c>
       <c r="B97">
@@ -13468,213 +13507,300 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98">
-        <f>2*(1-B98)</f>
-        <v>8.0000000000000071E-2</v>
+        <f t="shared" si="9"/>
+        <v>9.000000000000008E-2</v>
       </c>
       <c r="B98">
-        <v>0.96</v>
+        <v>0.95499999999999996</v>
       </c>
       <c r="C98">
         <f t="shared" si="4"/>
-        <v>0.55086734357186706</v>
+        <v>0.55494946009714197</v>
       </c>
       <c r="D98">
         <f t="shared" si="5"/>
-        <v>1.7506860712521695</v>
+        <v>1.6953977102721358</v>
       </c>
       <c r="E98">
         <f t="shared" si="6"/>
-        <v>3.1780538303479449</v>
+        <v>3.0550488507104094</v>
       </c>
       <c r="F98">
         <f t="shared" si="7"/>
-        <v>1.9915498973623778</v>
+        <v>1.9144679573924135</v>
       </c>
       <c r="G98" s="3">
         <f t="shared" si="8"/>
-        <v>0.13758253410786073</v>
+        <v>0.1292146649679701</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99">
         <f t="shared" si="9"/>
-        <v>6.0000000000000053E-2</v>
+        <v>8.0000000000000071E-2</v>
       </c>
       <c r="B99">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="C99">
         <f t="shared" si="4"/>
-        <v>0.54106450246968651</v>
+        <v>0.55086734357186706</v>
       </c>
       <c r="D99">
         <f t="shared" si="5"/>
-        <v>1.8807936081512504</v>
+        <v>1.7506860712521695</v>
       </c>
       <c r="E99">
         <f t="shared" si="6"/>
-        <v>3.4760986898352719</v>
+        <v>3.1780538303479449</v>
       </c>
       <c r="F99">
         <f t="shared" si="7"/>
-        <v>2.1783218153372172</v>
+        <v>1.9915498973623778</v>
       </c>
       <c r="G99" s="3">
         <f t="shared" si="8"/>
-        <v>0.15819290638616426</v>
+        <v>0.13758253410786073</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100">
         <f t="shared" si="9"/>
-        <v>5.0000000000000044E-2</v>
+        <v>7.0000000000000062E-2</v>
       </c>
       <c r="B100">
-        <v>0.97499999999999998</v>
+        <v>0.96499999999999997</v>
       </c>
       <c r="C100">
         <f t="shared" si="4"/>
-        <v>0.53498867327936173</v>
+        <v>0.54628605188867885</v>
       </c>
       <c r="D100">
         <f t="shared" si="5"/>
-        <v>1.9599639845400536</v>
+        <v>1.8119106729525971</v>
       </c>
       <c r="E100">
         <f t="shared" si="6"/>
-        <v>3.6635616461296454</v>
+        <v>3.3167800398495713</v>
       </c>
       <c r="F100">
         <f t="shared" si="7"/>
-        <v>2.2957968020105652</v>
+        <v>2.0784836571546679</v>
       </c>
       <c r="G100" s="3">
         <f t="shared" si="8"/>
-        <v>0.17134642275037609</v>
+        <v>0.1471225862187108</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101">
         <f t="shared" si="9"/>
-        <v>4.0000000000000036E-2</v>
+        <v>6.0000000000000053E-2</v>
       </c>
       <c r="B101">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="C101">
         <f t="shared" si="4"/>
-        <v>0.52770908040868747</v>
+        <v>0.54106450246968651</v>
       </c>
       <c r="D101">
         <f t="shared" si="5"/>
-        <v>2.0537489106318221</v>
+        <v>1.8807936081512504</v>
       </c>
       <c r="E101">
         <f t="shared" si="6"/>
-        <v>3.8918202981106256</v>
+        <v>3.4760986898352719</v>
       </c>
       <c r="F101">
         <f t="shared" si="7"/>
-        <v>2.4388366997567354</v>
+        <v>2.1783218153372172</v>
       </c>
       <c r="G101" s="3">
         <f t="shared" si="8"/>
-        <v>0.18750480505742237</v>
+        <v>0.15819290638616426</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102">
-        <f>2*(1-B102)</f>
-        <v>2.0000000000000018E-2</v>
+        <f t="shared" si="9"/>
+        <v>5.0000000000000044E-2</v>
       </c>
       <c r="B102">
-        <v>0.99</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="C102">
         <f t="shared" si="4"/>
-        <v>0.50626489621869231</v>
+        <v>0.53498867327936173</v>
       </c>
       <c r="D102">
         <f t="shared" si="5"/>
-        <v>2.3263478740408408</v>
+        <v>1.9599639845400536</v>
       </c>
       <c r="E102">
         <f t="shared" si="6"/>
-        <v>4.5951198501345889</v>
+        <v>3.6635616461296454</v>
       </c>
       <c r="F102">
         <f t="shared" si="7"/>
-        <v>2.8795643354163811</v>
+        <v>2.2957968020105652</v>
       </c>
       <c r="G102" s="3">
         <f t="shared" si="8"/>
-        <v>0.23780470132981851</v>
+        <v>0.17134642275037609</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103">
-        <f>2*(1-B103)</f>
-        <v>1.0000000000000009E-2</v>
+        <f t="shared" si="9"/>
+        <v>4.0000000000000036E-2</v>
       </c>
       <c r="B103">
-        <v>0.995</v>
+        <v>0.98</v>
       </c>
       <c r="C103">
         <f t="shared" si="4"/>
-        <v>0.48662024743359988</v>
+        <v>0.52770908040868747</v>
       </c>
       <c r="D103">
         <f t="shared" si="5"/>
-        <v>2.5758293035488999</v>
+        <v>2.0537489106318221</v>
       </c>
       <c r="E103">
         <f t="shared" si="6"/>
-        <v>5.2933048247244914</v>
+        <v>3.8918202981106256</v>
       </c>
       <c r="F103">
         <f t="shared" si="7"/>
-        <v>3.3170868849737754</v>
+        <v>2.4388366997567354</v>
       </c>
       <c r="G103" s="3">
         <f t="shared" si="8"/>
+        <v>0.18750480505742237</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <f t="shared" si="9"/>
+        <v>3.0000000000000027E-2</v>
+      </c>
+      <c r="B104">
+        <v>0.98499999999999999</v>
+      </c>
+      <c r="C104">
+        <f t="shared" si="4"/>
+        <v>0.51859074145320205</v>
+      </c>
+      <c r="D104">
+        <f t="shared" si="5"/>
+        <v>2.1700903775845601</v>
+      </c>
+      <c r="E104">
+        <f t="shared" si="6"/>
+        <v>4.1845914400698776</v>
+      </c>
+      <c r="F104">
+        <f t="shared" si="7"/>
+        <v>2.6223038053645027</v>
+      </c>
+      <c r="G104" s="3">
+        <f t="shared" si="8"/>
+        <v>0.2083846057523572</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A105">
+        <f>2*(1-B105)</f>
+        <v>2.0000000000000018E-2</v>
+      </c>
+      <c r="B105">
+        <v>0.99</v>
+      </c>
+      <c r="C105">
+        <f t="shared" si="4"/>
+        <v>0.50626489621869231</v>
+      </c>
+      <c r="D105">
+        <f t="shared" si="5"/>
+        <v>2.3263478740408408</v>
+      </c>
+      <c r="E105">
+        <f t="shared" si="6"/>
+        <v>4.5951198501345889</v>
+      </c>
+      <c r="F105">
+        <f t="shared" si="7"/>
+        <v>2.8795643354163811</v>
+      </c>
+      <c r="G105" s="3">
+        <f t="shared" si="8"/>
+        <v>0.23780470132981851</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A106">
+        <f>2*(1-B106)</f>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="B106">
+        <v>0.995</v>
+      </c>
+      <c r="C106">
+        <f t="shared" si="4"/>
+        <v>0.48662024743359988</v>
+      </c>
+      <c r="D106">
+        <f t="shared" si="5"/>
+        <v>2.5758293035488999</v>
+      </c>
+      <c r="E106">
+        <f t="shared" si="6"/>
+        <v>5.2933048247244914</v>
+      </c>
+      <c r="F106">
+        <f t="shared" si="7"/>
+        <v>3.3170868849737754</v>
+      </c>
+      <c r="G106" s="3">
+        <f t="shared" si="8"/>
         <v>0.28777434141446917</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B104">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B107">
         <v>1</v>
       </c>
-      <c r="D104" t="e">
+      <c r="D107" t="e">
         <f t="shared" si="5"/>
         <v>#NUM!</v>
       </c>
-      <c r="E104" t="e">
+      <c r="E107" t="e">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="F104" t="e">
+      <c r="F107" t="e">
         <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="G104" s="3" t="e">
+      <c r="G107" s="3" t="e">
         <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A106" s="12" t="s">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A109" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B106" s="12"/>
-      <c r="C106" s="12"/>
-      <c r="D106" s="12"/>
-      <c r="E106" s="12"/>
-      <c r="F106" s="12"/>
-      <c r="G106" s="12"/>
+      <c r="B109" s="14"/>
+      <c r="C109" s="14"/>
+      <c r="D109" s="14"/>
+      <c r="E109" s="14"/>
+      <c r="F109" s="14"/>
+      <c r="G109" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A106:G106"/>
+    <mergeCell ref="A109:G109"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>